<commit_message>
adjust plot names for barplots
adjust plot names for bar plots, so that the names are all "printed"
</commit_message>
<xml_diff>
--- a/inst/extdata/misa_data/misa_scenarios.xlsx
+++ b/inst/extdata/misa_data/misa_scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pschue\Documents\R\git\kwb.misa\inst\extdata\misa_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97AFF7BD-EAF8-4409-9E93-C1ACD69BECF0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C90754B5-4D12-4554-9691-983EC0FF2F0B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -193,25 +193,25 @@
     <t xml:space="preserve">misa_sccenario_no </t>
   </si>
   <si>
-    <t>Straßen 10a</t>
-  </si>
-  <si>
-    <t>Liegen. 10a</t>
-  </si>
-  <si>
-    <t>Straßen 30a</t>
-  </si>
-  <si>
-    <t>Liegen. 30a</t>
-  </si>
-  <si>
-    <t>Str. + Lieg. 10a</t>
-  </si>
-  <si>
-    <t>Str. + Lieg.30a</t>
-  </si>
-  <si>
-    <t>Str. + Lieg. &gt;30a</t>
+    <t>Str10a</t>
+  </si>
+  <si>
+    <t>Lieg10a</t>
+  </si>
+  <si>
+    <t>Str30a</t>
+  </si>
+  <si>
+    <t>Lieg30a</t>
+  </si>
+  <si>
+    <t>StrLieg10a</t>
+  </si>
+  <si>
+    <t>StrLieg30a</t>
+  </si>
+  <si>
+    <t>StrLieg&gt;30a</t>
   </si>
 </sst>
 </file>

</xml_diff>